<commit_message>
uploaded Venues data file
</commit_message>
<xml_diff>
--- a/Data1.xlsx
+++ b/Data1.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="178">
   <si>
     <t xml:space="preserve">Sr No</t>
   </si>
@@ -92,13 +92,28 @@
     <t xml:space="preserve">Class Room</t>
   </si>
   <si>
+    <t xml:space="preserve">Aryan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arnav.prasad.tech@gmail.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Academic Complex 102</t>
   </si>
   <si>
+    <t xml:space="preserve">Keshav</t>
+  </si>
+  <si>
     <t xml:space="preserve">Academic Complex 103</t>
   </si>
   <si>
+    <t xml:space="preserve">Atharva</t>
+  </si>
+  <si>
     <t xml:space="preserve">Academic Complex 104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idris</t>
   </si>
   <si>
     <t xml:space="preserve">2nd floor</t>
@@ -967,7 +982,7 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>2837160</xdr:colOff>
       <xdr:row>122</xdr:row>
-      <xdr:rowOff>150480</xdr:rowOff>
+      <xdr:rowOff>150840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -980,7 +995,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11862000" y="22330800"/>
+          <a:off x="11862000" y="22254840"/>
           <a:ext cx="4695480" cy="3046320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1087,7 +1102,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
         <v>20</v>
       </c>
@@ -1119,19 +1134,25 @@
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
+      <c r="O2" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
+      <c r="Q2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="S2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3"/>
       <c r="C3" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>22</v>
@@ -1155,19 +1176,27 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="O3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>1231231231</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="S3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3"/>
       <c r="C4" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>22</v>
@@ -1191,19 +1220,27 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
+      <c r="O4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>2342342342</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="S4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3"/>
       <c r="C5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>22</v>
@@ -1227,13 +1264,21 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
+      <c r="O5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>6546546546</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="S5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3"/>
       <c r="J6" s="10"/>
       <c r="K6" s="3"/>
@@ -1241,18 +1286,22 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
+      <c r="P6" s="3" t="n">
+        <v>7878787878</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3"/>
       <c r="C7" s="9" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>22</v>
@@ -1285,10 +1334,10 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3"/>
       <c r="C8" s="9" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>22</v>
@@ -1321,10 +1370,10 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3"/>
       <c r="C9" s="9" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>22</v>
@@ -1357,10 +1406,10 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3"/>
       <c r="C10" s="9" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>22</v>
@@ -1434,10 +1483,10 @@
         <v>2</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
@@ -1463,13 +1512,13 @@
       <c r="A15" s="19"/>
       <c r="B15" s="20"/>
       <c r="C15" s="19" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>1</v>
@@ -1487,32 +1536,32 @@
         <v>60</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="M15" s="20" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N15" s="20" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="O15" s="24" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="Q15" s="17"/>
       <c r="R15" s="17" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="S15" s="17" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="T15" s="17" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="U15" s="18"/>
       <c r="V15" s="18"/>
@@ -1536,7 +1585,7 @@
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J17" s="10"/>
       <c r="K17" s="3"/>
@@ -1552,13 +1601,13 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3"/>
       <c r="C18" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>1</v>
@@ -1586,13 +1635,13 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3"/>
       <c r="C19" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>1</v>
@@ -1620,13 +1669,13 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3"/>
       <c r="C20" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>1</v>
@@ -1654,13 +1703,13 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3"/>
       <c r="C21" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F21" s="1" t="n">
         <v>1</v>
@@ -1688,13 +1737,13 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="3"/>
       <c r="C22" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>1</v>
@@ -1750,10 +1799,10 @@
         <v>4</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
@@ -1776,13 +1825,13 @@
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11"/>
       <c r="B26" s="25" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>22</v>
@@ -1803,38 +1852,38 @@
         <v>72</v>
       </c>
       <c r="K26" s="26" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="L26" s="27" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="M26" s="28" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N26" s="16" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="O26" s="29" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="P26" s="16"/>
       <c r="Q26" s="16"/>
       <c r="R26" s="16"/>
       <c r="S26" s="16"/>
       <c r="T26" s="16" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11"/>
       <c r="B27" s="25" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>22</v>
@@ -1855,38 +1904,38 @@
         <v>72</v>
       </c>
       <c r="K27" s="26" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="L27" s="30" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M27" s="28" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N27" s="16" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="O27" s="29" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="P27" s="16"/>
       <c r="Q27" s="16"/>
       <c r="R27" s="16"/>
       <c r="S27" s="16"/>
       <c r="T27" s="16" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11"/>
       <c r="B28" s="25" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>22</v>
@@ -1907,26 +1956,26 @@
         <v>72</v>
       </c>
       <c r="K28" s="26" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="L28" s="27" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="M28" s="28" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N28" s="16" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="O28" s="29" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="P28" s="16"/>
       <c r="Q28" s="16"/>
       <c r="R28" s="16"/>
       <c r="S28" s="16"/>
       <c r="T28" s="16" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1948,7 +1997,7 @@
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="9" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="J30" s="10"/>
       <c r="K30" s="3"/>
@@ -1963,16 +2012,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="31" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F31" s="11" t="n">
         <v>1</v>
@@ -1990,19 +2039,19 @@
         <v>40</v>
       </c>
       <c r="K31" s="28" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="M31" s="29" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N31" s="16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O31" s="28" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="P31" s="16"/>
       <c r="Q31" s="16"/>
@@ -2013,7 +2062,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="31"/>
       <c r="C32" s="11" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>22</v>
@@ -2037,19 +2086,19 @@
         <v>60</v>
       </c>
       <c r="K32" s="28" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="L32" s="32" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M32" s="29" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N32" s="16" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="O32" s="28" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="P32" s="16"/>
       <c r="Q32" s="16"/>
@@ -2060,13 +2109,13 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="31"/>
       <c r="C33" s="11" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F33" s="11" t="n">
         <v>1</v>
@@ -2084,19 +2133,19 @@
         <v>40</v>
       </c>
       <c r="K33" s="28" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="L33" s="16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="M33" s="29" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="N33" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="O33" s="28" t="s">
         <v>72</v>
-      </c>
-      <c r="O33" s="28" t="s">
-        <v>67</v>
       </c>
       <c r="P33" s="16"/>
       <c r="Q33" s="16"/>
@@ -2149,7 +2198,7 @@
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="J37" s="10"/>
       <c r="K37" s="3"/>
@@ -2165,13 +2214,13 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="3"/>
       <c r="C38" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F38" s="1" t="n">
         <v>1</v>
@@ -2190,7 +2239,7 @@
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="33" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
@@ -2203,7 +2252,7 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3"/>
       <c r="C39" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D39" s="9" t="s">
         <v>22</v>
@@ -2227,10 +2276,10 @@
         <v>30</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L39" s="33" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
@@ -2281,10 +2330,10 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="3"/>
       <c r="C42" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E42" s="9" t="s">
         <v>22</v>
@@ -2306,7 +2355,7 @@
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="33" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
@@ -2319,7 +2368,7 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="3"/>
       <c r="D43" s="9" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>22</v>
@@ -2341,7 +2390,7 @@
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="33" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
@@ -2367,13 +2416,13 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3"/>
       <c r="C45" s="9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F45" s="1" t="n">
         <v>1</v>
@@ -2391,10 +2440,10 @@
         <v>40</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L45" s="33" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
@@ -2420,10 +2469,10 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="3"/>
       <c r="C47" s="9" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>22</v>
@@ -2444,10 +2493,10 @@
         <v>80</v>
       </c>
       <c r="K47" s="16" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L47" s="33" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
@@ -2476,7 +2525,7 @@
       </c>
       <c r="B49" s="3"/>
       <c r="C49" s="9" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="J49" s="10"/>
       <c r="K49" s="3"/>
@@ -2492,7 +2541,7 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3"/>
       <c r="C50" s="34" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="11"/>
@@ -2514,13 +2563,13 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="3"/>
       <c r="C51" s="11" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F51" s="11" t="n">
         <v>1</v>
@@ -2532,10 +2581,10 @@
         <v>90</v>
       </c>
       <c r="K51" s="16" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="L51" s="32" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="M51" s="3"/>
       <c r="N51" s="3"/>
@@ -2548,13 +2597,13 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="3"/>
       <c r="C52" s="11" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F52" s="11" t="n">
         <v>1</v>
@@ -2566,10 +2615,10 @@
         <v>120</v>
       </c>
       <c r="K52" s="16" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="L52" s="32" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="M52" s="3"/>
       <c r="N52" s="3"/>
@@ -2582,13 +2631,13 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="3"/>
       <c r="C53" s="11" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D53" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E53" s="11" t="s">
         <v>96</v>
-      </c>
-      <c r="E53" s="11" t="s">
-        <v>91</v>
       </c>
       <c r="F53" s="11" t="n">
         <v>1</v>
@@ -2600,10 +2649,10 @@
         <v>120</v>
       </c>
       <c r="K53" s="16" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="L53" s="32" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
@@ -2616,13 +2665,13 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="3"/>
       <c r="C54" s="11" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="F54" s="11" t="n">
         <v>1</v>
@@ -2634,7 +2683,7 @@
         <v>15</v>
       </c>
       <c r="K54" s="16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L54" s="16"/>
       <c r="M54" s="3"/>
@@ -2648,13 +2697,13 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="3"/>
       <c r="C55" s="11" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F55" s="11" t="n">
         <v>1</v>
@@ -2672,10 +2721,10 @@
         <v>30</v>
       </c>
       <c r="K55" s="16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L55" s="32" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M55" s="3"/>
       <c r="N55" s="3"/>
@@ -2688,13 +2737,13 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="3"/>
       <c r="C56" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F56" s="11" t="n">
         <v>1</v>
@@ -2712,10 +2761,10 @@
         <v>90</v>
       </c>
       <c r="K56" s="16" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="L56" s="32" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="M56" s="3"/>
       <c r="N56" s="3"/>
@@ -2728,13 +2777,13 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="3"/>
       <c r="C57" s="11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D57" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E57" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="E57" s="11" t="s">
-        <v>101</v>
       </c>
       <c r="F57" s="11" t="n">
         <v>1</v>
@@ -2752,10 +2801,10 @@
         <v>40</v>
       </c>
       <c r="K57" s="16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L57" s="32" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
@@ -2791,7 +2840,7 @@
       </c>
       <c r="B59" s="3"/>
       <c r="C59" s="34" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D59" s="11"/>
       <c r="E59" s="11"/>
@@ -2813,13 +2862,13 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="3"/>
       <c r="C60" s="11" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F60" s="11" t="n">
         <v>1</v>
@@ -2837,10 +2886,10 @@
         <v>36</v>
       </c>
       <c r="K60" s="16" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="L60" s="32" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="M60" s="3"/>
       <c r="N60" s="3"/>
@@ -2853,13 +2902,13 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="3"/>
       <c r="C61" s="11" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F61" s="11" t="n">
         <v>1</v>
@@ -2877,10 +2926,10 @@
         <v>18</v>
       </c>
       <c r="K61" s="16" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="L61" s="32" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M61" s="3"/>
       <c r="N61" s="3"/>
@@ -2893,13 +2942,13 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="3"/>
       <c r="C62" s="11" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F62" s="11" t="n">
         <v>1</v>
@@ -2917,10 +2966,10 @@
         <v>18</v>
       </c>
       <c r="K62" s="16" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="L62" s="32" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="M62" s="3"/>
       <c r="N62" s="3"/>
@@ -2933,10 +2982,10 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="3"/>
       <c r="C63" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E63" s="11"/>
       <c r="F63" s="11" t="n">
@@ -2955,10 +3004,10 @@
         <v>180</v>
       </c>
       <c r="K63" s="16" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L63" s="32" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="M63" s="3"/>
       <c r="N63" s="3"/>
@@ -2987,7 +3036,7 @@
       </c>
       <c r="B65" s="3"/>
       <c r="C65" s="40" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="J65" s="10"/>
       <c r="K65" s="3"/>
@@ -3003,13 +3052,13 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="3"/>
       <c r="C66" s="9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F66" s="1" t="n">
         <v>1</v>
@@ -3027,10 +3076,10 @@
         <v>100</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="L66" s="33" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M66" s="3"/>
       <c r="N66" s="3"/>
@@ -3043,13 +3092,13 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="3"/>
       <c r="C67" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F67" s="1" t="n">
         <v>1</v>
@@ -3067,10 +3116,10 @@
         <v>120</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L67" s="33" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M67" s="3"/>
       <c r="N67" s="3"/>
@@ -3083,13 +3132,13 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="3"/>
       <c r="C68" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="F68" s="1" t="n">
         <v>1</v>
@@ -3107,10 +3156,10 @@
         <v>50</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L68" s="33" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M68" s="3"/>
       <c r="N68" s="3"/>
@@ -3123,13 +3172,13 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="3"/>
       <c r="C69" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>1</v>
@@ -3147,10 +3196,10 @@
         <v>50</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L69" s="33" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M69" s="3"/>
       <c r="N69" s="3"/>
@@ -3163,13 +3212,13 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="3"/>
       <c r="C70" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F70" s="1" t="n">
         <v>1</v>
@@ -3187,10 +3236,10 @@
         <v>105</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L70" s="33" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M70" s="3"/>
       <c r="N70" s="3"/>
@@ -3203,13 +3252,13 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="3"/>
       <c r="C71" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F71" s="1" t="n">
         <v>1</v>
@@ -3227,10 +3276,10 @@
         <v>40</v>
       </c>
       <c r="K71" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L71" s="33" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M71" s="3"/>
       <c r="N71" s="3"/>
@@ -3259,7 +3308,7 @@
       </c>
       <c r="B73" s="3"/>
       <c r="C73" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="J73" s="10"/>
       <c r="K73" s="3"/>
@@ -3275,10 +3324,10 @@
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="3"/>
       <c r="C74" s="9" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>1</v>
@@ -3294,7 +3343,7 @@
       </c>
       <c r="J74" s="10"/>
       <c r="K74" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="L74" s="3"/>
       <c r="M74" s="3"/>
@@ -3308,7 +3357,7 @@
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="3"/>
       <c r="E75" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F75" s="1" t="n">
         <v>1</v>
@@ -3324,7 +3373,7 @@
       </c>
       <c r="J75" s="10"/>
       <c r="K75" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L75" s="3"/>
       <c r="M75" s="3"/>
@@ -3338,13 +3387,13 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="3"/>
       <c r="C76" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F76" s="1" t="n">
         <v>1</v>
@@ -3362,34 +3411,34 @@
         <v>25</v>
       </c>
       <c r="K76" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L76" s="33" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="N76" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="O76" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="P76" s="3"/>
       <c r="Q76" s="41" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R76" s="3"/>
       <c r="S76" s="3"/>
       <c r="T76" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="3"/>
       <c r="E77" s="9" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F77" s="1" t="n">
         <v>1</v>
@@ -3405,7 +3454,7 @@
       </c>
       <c r="J77" s="10"/>
       <c r="K77" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="L77" s="3"/>
       <c r="M77" s="3"/>
@@ -3419,13 +3468,13 @@
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="3"/>
       <c r="C78" s="9" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>1</v>
@@ -3443,40 +3492,40 @@
         <v>20</v>
       </c>
       <c r="K78" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="L78" s="33" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="N78" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="O78" s="3" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="P78" s="3"/>
       <c r="Q78" s="41" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="R78" s="3"/>
       <c r="S78" s="3"/>
       <c r="T78" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="3"/>
       <c r="C79" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>2</v>
@@ -3494,14 +3543,14 @@
         <v>60</v>
       </c>
       <c r="K79" s="3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="L79" s="3"/>
       <c r="M79" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="N79" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="O79" s="3"/>
       <c r="P79" s="3"/>
@@ -3512,16 +3561,16 @@
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="3"/>
       <c r="D80" s="9" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="J80" s="10" t="n">
         <v>60</v>
       </c>
       <c r="K80" s="3" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="L80" s="33" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="M80" s="3"/>
       <c r="N80" s="3"/>
@@ -3534,13 +3583,13 @@
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="3"/>
       <c r="C81" s="9" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>1</v>
@@ -3558,23 +3607,23 @@
         <v>25</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="L81" s="33" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="N81" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="O81" s="3" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="P81" s="3"/>
       <c r="Q81" s="41" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="R81" s="3"/>
       <c r="S81" s="3"/>
@@ -3610,7 +3659,7 @@
       </c>
       <c r="B83" s="3"/>
       <c r="C83" s="9" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="J83" s="10"/>
       <c r="K83" s="3"/>
@@ -3626,10 +3675,10 @@
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="3"/>
       <c r="C84" s="9" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E84" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F84" s="1" t="n">
         <v>1</v>
@@ -3657,7 +3706,7 @@
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3"/>
       <c r="D85" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F85" s="1" t="n">
         <v>1</v>
@@ -3710,7 +3759,7 @@
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3"/>
       <c r="E87" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F87" s="1" t="n">
         <v>1</v>
@@ -3738,7 +3787,7 @@
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="3"/>
       <c r="C88" s="9" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="F88" s="1" t="n">
         <v>1</v>
@@ -3766,10 +3815,10 @@
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="3"/>
       <c r="C89" s="9" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F89" s="1" t="n">
         <v>2</v>
@@ -3797,13 +3846,13 @@
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="3"/>
       <c r="C90" s="9" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E90" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F90" s="1" t="n">
         <v>1</v>
@@ -3831,13 +3880,13 @@
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="3"/>
       <c r="C91" s="9" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D91" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F91" s="1" t="n">
         <v>1</v>
@@ -3865,7 +3914,7 @@
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="3"/>
       <c r="D92" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J92" s="10"/>
       <c r="K92" s="3"/>
@@ -3884,7 +3933,7 @@
       </c>
       <c r="B93" s="3"/>
       <c r="C93" s="9" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="J93" s="10"/>
       <c r="K93" s="3"/>
@@ -3913,7 +3962,7 @@
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="3"/>
       <c r="C95" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>22</v>
@@ -3944,7 +3993,7 @@
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="3"/>
       <c r="C96" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E96" s="9" t="s">
         <v>22</v>
@@ -3975,7 +4024,7 @@
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="3"/>
       <c r="C97" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>22</v>
@@ -4031,10 +4080,10 @@
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="3"/>
       <c r="C99" s="9" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="F99" s="1" t="n">
         <v>1</v>
@@ -4066,42 +4115,47 @@
     <mergeCell ref="B31:B33"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="L15" r:id="rId1" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EXHWOoyhaSxHm7Lao21I5xQBIQJnC9zkwJAsWTPrz0VqbQ?e=iPwYTM"/>
-    <hyperlink ref="L26" r:id="rId2" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EY7XfX1KNQlMkCTxXJQI0BABleLdKq1eLj2eJ2QNIOqH1A?e=GsPQog"/>
-    <hyperlink ref="L27" r:id="rId3" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EfGEwf925gBLsi9eaW-g3ykBCPS2_nS6iGvPHJ5mHA9sng?e=W93FeG"/>
-    <hyperlink ref="L28" r:id="rId4" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="L31" r:id="rId5" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=FfvEO4"/>
-    <hyperlink ref="L32" r:id="rId6" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/EQV193k-k_pNq0ihEG9vBHIBUbOPsCqlm1XRtDJ9Dwq6qw?e=qgBbbB"/>
-    <hyperlink ref="L33" r:id="rId7" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=yIhjgd"/>
-    <hyperlink ref="L38" r:id="rId8" display="Fluid Mechanics_Basement1.jpg"/>
-    <hyperlink ref="L39" r:id="rId9" display="App Mechanics_First Floor_Classroom.jpg"/>
-    <hyperlink ref="L42" r:id="rId10" display="App Mechanics_Classroom2.jpg"/>
-    <hyperlink ref="L43" r:id="rId11" display="App Mechanics Classroom1 (1).jpg"/>
-    <hyperlink ref="L45" r:id="rId12" display="App Mech Ground Floor Seminar Hall.jpg"/>
-    <hyperlink ref="L47" r:id="rId13" display="R22.jpg"/>
-    <hyperlink ref="L51" r:id="rId14" display="https://drive.google.com/file/d/11r8JUGcdvTO0ylOI_nn1YEYv9b4CKOKq/view?usp=sharing"/>
-    <hyperlink ref="L52" r:id="rId15" display="https://drive.google.com/file/d/1xfCJ7OavNoyQdfRC-VI19CAZpL4tOAEL/view?usp=sharing"/>
-    <hyperlink ref="L53" r:id="rId16" display="https://drive.google.com/file/d/1WSBvMorlthEbWyaCh8JdxRMas7G4kjVu/view?usp=sharing"/>
-    <hyperlink ref="L55" r:id="rId17" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
-    <hyperlink ref="L56" r:id="rId18" display="https://drive.google.com/file/d/1E-q97N6HQpt942F05ddKGT_D6nsHbDe_/view?usp=sharing"/>
-    <hyperlink ref="L57" r:id="rId19" display="https://drive.google.com/file/d/1orGoTWToL2cNbFSvNjVnGiJBTqj4-x7p/view?usp=sharing"/>
-    <hyperlink ref="L60" r:id="rId20" display="https://drive.google.com/file/d/1bJecDqhyMaVv0s9jZLgIDUpY1PGb-2qw/view?usp=sharing"/>
-    <hyperlink ref="L61" r:id="rId21" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
-    <hyperlink ref="L62" r:id="rId22" display="https://drive.google.com/file/d/1V56Qmp1d-mKg5U3SGllOvQp56yiec8hE/view?usp=sharing"/>
-    <hyperlink ref="L63" r:id="rId23" display="https://drive.google.com/file/d/1pcndMBRukVQKbKa81_jG_82Q2cZywHFu/view?usp=sharing"/>
-    <hyperlink ref="L66" r:id="rId24" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L67" r:id="rId25" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L68" r:id="rId26" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L69" r:id="rId27" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L70" r:id="rId28" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L71" r:id="rId29" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L76" r:id="rId30" display="Env Classroom.jpeg"/>
-    <hyperlink ref="Q76" r:id="rId31" display="muk.civil@coep.ac.in"/>
-    <hyperlink ref="L78" r:id="rId32" display="CM Classroom.jpeg"/>
-    <hyperlink ref="Q78" r:id="rId33" display="gsv.civil@coeptech.ac.in"/>
-    <hyperlink ref="L80" r:id="rId34" display="R8.jpeg"/>
-    <hyperlink ref="L81" r:id="rId35" display="Geotech Classroom.jpeg"/>
-    <hyperlink ref="Q81" r:id="rId36" display="yak.civl@coeptech.ac.in"/>
+    <hyperlink ref="Q2" r:id="rId1" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="Q3" r:id="rId2" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="Q4" r:id="rId3" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="Q5" r:id="rId4" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="Q6" r:id="rId5" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="L15" r:id="rId6" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EXHWOoyhaSxHm7Lao21I5xQBIQJnC9zkwJAsWTPrz0VqbQ?e=iPwYTM"/>
+    <hyperlink ref="L26" r:id="rId7" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EY7XfX1KNQlMkCTxXJQI0BABleLdKq1eLj2eJ2QNIOqH1A?e=GsPQog"/>
+    <hyperlink ref="L27" r:id="rId8" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EfGEwf925gBLsi9eaW-g3ykBCPS2_nS6iGvPHJ5mHA9sng?e=W93FeG"/>
+    <hyperlink ref="L28" r:id="rId9" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
+    <hyperlink ref="L31" r:id="rId10" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=FfvEO4"/>
+    <hyperlink ref="L32" r:id="rId11" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/EQV193k-k_pNq0ihEG9vBHIBUbOPsCqlm1XRtDJ9Dwq6qw?e=qgBbbB"/>
+    <hyperlink ref="L33" r:id="rId12" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=yIhjgd"/>
+    <hyperlink ref="L38" r:id="rId13" display="Fluid Mechanics_Basement1.jpg"/>
+    <hyperlink ref="L39" r:id="rId14" display="App Mechanics_First Floor_Classroom.jpg"/>
+    <hyperlink ref="L42" r:id="rId15" display="App Mechanics_Classroom2.jpg"/>
+    <hyperlink ref="L43" r:id="rId16" display="App Mechanics Classroom1 (1).jpg"/>
+    <hyperlink ref="L45" r:id="rId17" display="App Mech Ground Floor Seminar Hall.jpg"/>
+    <hyperlink ref="L47" r:id="rId18" display="R22.jpg"/>
+    <hyperlink ref="L51" r:id="rId19" display="https://drive.google.com/file/d/11r8JUGcdvTO0ylOI_nn1YEYv9b4CKOKq/view?usp=sharing"/>
+    <hyperlink ref="L52" r:id="rId20" display="https://drive.google.com/file/d/1xfCJ7OavNoyQdfRC-VI19CAZpL4tOAEL/view?usp=sharing"/>
+    <hyperlink ref="L53" r:id="rId21" display="https://drive.google.com/file/d/1WSBvMorlthEbWyaCh8JdxRMas7G4kjVu/view?usp=sharing"/>
+    <hyperlink ref="L55" r:id="rId22" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
+    <hyperlink ref="L56" r:id="rId23" display="https://drive.google.com/file/d/1E-q97N6HQpt942F05ddKGT_D6nsHbDe_/view?usp=sharing"/>
+    <hyperlink ref="L57" r:id="rId24" display="https://drive.google.com/file/d/1orGoTWToL2cNbFSvNjVnGiJBTqj4-x7p/view?usp=sharing"/>
+    <hyperlink ref="L60" r:id="rId25" display="https://drive.google.com/file/d/1bJecDqhyMaVv0s9jZLgIDUpY1PGb-2qw/view?usp=sharing"/>
+    <hyperlink ref="L61" r:id="rId26" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
+    <hyperlink ref="L62" r:id="rId27" display="https://drive.google.com/file/d/1V56Qmp1d-mKg5U3SGllOvQp56yiec8hE/view?usp=sharing"/>
+    <hyperlink ref="L63" r:id="rId28" display="https://drive.google.com/file/d/1pcndMBRukVQKbKa81_jG_82Q2cZywHFu/view?usp=sharing"/>
+    <hyperlink ref="L66" r:id="rId29" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L67" r:id="rId30" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L68" r:id="rId31" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L69" r:id="rId32" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L70" r:id="rId33" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L71" r:id="rId34" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L76" r:id="rId35" display="Env Classroom.jpeg"/>
+    <hyperlink ref="Q76" r:id="rId36" display="muk.civil@coep.ac.in"/>
+    <hyperlink ref="L78" r:id="rId37" display="CM Classroom.jpeg"/>
+    <hyperlink ref="Q78" r:id="rId38" display="gsv.civil@coeptech.ac.in"/>
+    <hyperlink ref="L80" r:id="rId39" display="R8.jpeg"/>
+    <hyperlink ref="L81" r:id="rId40" display="Geotech Classroom.jpeg"/>
+    <hyperlink ref="Q81" r:id="rId41" display="yak.civl@coeptech.ac.in"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4110,7 +4164,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId37"/>
+  <drawing r:id="rId42"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
uploaded venue data file version2
</commit_message>
<xml_diff>
--- a/Data1.xlsx
+++ b/Data1.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="178">
   <si>
     <t xml:space="preserve">Sr No</t>
   </si>
@@ -1147,7 +1147,9 @@
       <c r="S2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="3"/>
+      <c r="B3" s="9" t="s">
+        <v>20</v>
+      </c>
       <c r="C3" s="9" t="n">
         <v>1</v>
       </c>
@@ -1191,7 +1193,9 @@
       <c r="S3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3"/>
+      <c r="B4" s="9" t="s">
+        <v>20</v>
+      </c>
       <c r="C4" s="9" t="n">
         <v>1</v>
       </c>
@@ -1235,7 +1239,9 @@
       <c r="S4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3"/>
+      <c r="B5" s="9" t="s">
+        <v>20</v>
+      </c>
       <c r="C5" s="9" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Uploaded Venue data version3
</commit_message>
<xml_diff>
--- a/Data1.xlsx
+++ b/Data1.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="180">
   <si>
     <t xml:space="preserve">Sr No</t>
   </si>
@@ -83,6 +83,9 @@
     <t xml:space="preserve">Campus (North/South)</t>
   </si>
   <si>
+    <t xml:space="preserve">Venue Admin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Academic Complex Building</t>
   </si>
   <si>
@@ -96,6 +99,9 @@
   </si>
   <si>
     <t xml:space="preserve">arnav.prasad.tech@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arnav.davpune@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Academic Complex 102</t>
@@ -1038,6 +1044,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="30.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="35.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="3" width="28.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="29.03"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="true" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1101,19 +1108,22 @@
       <c r="T1" s="5" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>4</v>
@@ -1135,29 +1145,32 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="S2" s="3"/>
+      <c r="U2" s="0" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>4</v>
@@ -1179,31 +1192,34 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="P3" s="3" t="n">
         <v>1231231231</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="S3" s="3"/>
+      <c r="U3" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="S3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>4</v>
@@ -1225,31 +1241,34 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="P4" s="3" t="n">
         <v>2342342342</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="S4" s="3"/>
+      <c r="U4" s="0" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>4</v>
@@ -1271,18 +1290,21 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="P5" s="3" t="n">
         <v>6546546546</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="S5" s="3"/>
+      <c r="U5" s="0" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3"/>
@@ -1296,7 +1318,7 @@
         <v>7878787878</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
@@ -1304,13 +1326,13 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3"/>
       <c r="C7" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>4</v>
@@ -1340,13 +1362,13 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3"/>
       <c r="C8" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>4</v>
@@ -1376,13 +1398,13 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3"/>
       <c r="C9" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>4</v>
@@ -1412,13 +1434,13 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3"/>
       <c r="C10" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>4</v>
@@ -1489,10 +1511,10 @@
         <v>2</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
@@ -1518,13 +1540,13 @@
       <c r="A15" s="19"/>
       <c r="B15" s="20"/>
       <c r="C15" s="19" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>1</v>
@@ -1542,32 +1564,32 @@
         <v>60</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M15" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N15" s="20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O15" s="24" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="Q15" s="17"/>
       <c r="R15" s="17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="S15" s="17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="T15" s="17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="U15" s="18"/>
       <c r="V15" s="18"/>
@@ -1591,7 +1613,7 @@
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J17" s="10"/>
       <c r="K17" s="3"/>
@@ -1607,13 +1629,13 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3"/>
       <c r="C18" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>1</v>
@@ -1641,13 +1663,13 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3"/>
       <c r="C19" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>1</v>
@@ -1675,13 +1697,13 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3"/>
       <c r="C20" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>1</v>
@@ -1709,13 +1731,13 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3"/>
       <c r="C21" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F21" s="1" t="n">
         <v>1</v>
@@ -1743,13 +1765,13 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="3"/>
       <c r="C22" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>1</v>
@@ -1805,10 +1827,10 @@
         <v>4</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
@@ -1831,16 +1853,16 @@
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11"/>
       <c r="B26" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F26" s="11" t="n">
         <v>4</v>
@@ -1858,41 +1880,41 @@
         <v>72</v>
       </c>
       <c r="K26" s="26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L26" s="27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M26" s="28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N26" s="16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O26" s="29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="P26" s="16"/>
       <c r="Q26" s="16"/>
       <c r="R26" s="16"/>
       <c r="S26" s="16"/>
       <c r="T26" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11"/>
       <c r="B27" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F27" s="11" t="n">
         <v>4</v>
@@ -1910,41 +1932,41 @@
         <v>72</v>
       </c>
       <c r="K27" s="26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L27" s="30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M27" s="28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N27" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="O27" s="29" t="s">
         <v>63</v>
-      </c>
-      <c r="O27" s="29" t="s">
-        <v>61</v>
       </c>
       <c r="P27" s="16"/>
       <c r="Q27" s="16"/>
       <c r="R27" s="16"/>
       <c r="S27" s="16"/>
       <c r="T27" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11"/>
       <c r="B28" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F28" s="11" t="n">
         <v>4</v>
@@ -1962,26 +1984,26 @@
         <v>72</v>
       </c>
       <c r="K28" s="26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L28" s="27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M28" s="28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N28" s="16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="O28" s="29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="P28" s="16"/>
       <c r="Q28" s="16"/>
       <c r="R28" s="16"/>
       <c r="S28" s="16"/>
       <c r="T28" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2003,7 +2025,7 @@
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J30" s="10"/>
       <c r="K30" s="3"/>
@@ -2018,16 +2040,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="31" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F31" s="11" t="n">
         <v>1</v>
@@ -2045,19 +2067,19 @@
         <v>40</v>
       </c>
       <c r="K31" s="28" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M31" s="29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N31" s="16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O31" s="28" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="P31" s="16"/>
       <c r="Q31" s="16"/>
@@ -2068,13 +2090,13 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="31"/>
       <c r="C32" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F32" s="11" t="n">
         <v>1</v>
@@ -2092,19 +2114,19 @@
         <v>60</v>
       </c>
       <c r="K32" s="28" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L32" s="32" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="M32" s="29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N32" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="O32" s="28" t="s">
         <v>74</v>
-      </c>
-      <c r="O32" s="28" t="s">
-        <v>72</v>
       </c>
       <c r="P32" s="16"/>
       <c r="Q32" s="16"/>
@@ -2115,13 +2137,13 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="31"/>
       <c r="C33" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F33" s="11" t="n">
         <v>1</v>
@@ -2139,19 +2161,19 @@
         <v>40</v>
       </c>
       <c r="K33" s="28" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L33" s="16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M33" s="29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N33" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O33" s="28" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="P33" s="16"/>
       <c r="Q33" s="16"/>
@@ -2204,7 +2226,7 @@
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J37" s="10"/>
       <c r="K37" s="3"/>
@@ -2220,13 +2242,13 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="3"/>
       <c r="C38" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F38" s="1" t="n">
         <v>1</v>
@@ -2245,7 +2267,7 @@
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="33" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
@@ -2258,13 +2280,13 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3"/>
       <c r="C39" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F39" s="1" t="n">
         <v>1</v>
@@ -2282,10 +2304,10 @@
         <v>30</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L39" s="33" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
@@ -2336,13 +2358,13 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="3"/>
       <c r="C42" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F42" s="1" t="n">
         <v>1</v>
@@ -2361,7 +2383,7 @@
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="33" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
@@ -2374,10 +2396,10 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="3"/>
       <c r="D43" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F43" s="1" t="n">
         <v>1</v>
@@ -2396,7 +2418,7 @@
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="33" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
@@ -2422,13 +2444,13 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3"/>
       <c r="C45" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F45" s="1" t="n">
         <v>1</v>
@@ -2446,10 +2468,10 @@
         <v>40</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L45" s="33" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
@@ -2475,13 +2497,13 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="3"/>
       <c r="C47" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F47" s="1" t="n">
         <v>1</v>
@@ -2499,10 +2521,10 @@
         <v>80</v>
       </c>
       <c r="K47" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L47" s="33" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
@@ -2531,7 +2553,7 @@
       </c>
       <c r="B49" s="3"/>
       <c r="C49" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J49" s="10"/>
       <c r="K49" s="3"/>
@@ -2547,7 +2569,7 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3"/>
       <c r="C50" s="34" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="11"/>
@@ -2569,13 +2591,13 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="3"/>
       <c r="C51" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F51" s="11" t="n">
         <v>1</v>
@@ -2587,10 +2609,10 @@
         <v>90</v>
       </c>
       <c r="K51" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L51" s="32" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M51" s="3"/>
       <c r="N51" s="3"/>
@@ -2603,13 +2625,13 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="3"/>
       <c r="C52" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F52" s="11" t="n">
         <v>1</v>
@@ -2621,10 +2643,10 @@
         <v>120</v>
       </c>
       <c r="K52" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L52" s="32" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M52" s="3"/>
       <c r="N52" s="3"/>
@@ -2637,13 +2659,13 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="3"/>
       <c r="C53" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F53" s="11" t="n">
         <v>1</v>
@@ -2655,10 +2677,10 @@
         <v>120</v>
       </c>
       <c r="K53" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L53" s="32" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
@@ -2671,13 +2693,13 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="3"/>
       <c r="C54" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F54" s="11" t="n">
         <v>1</v>
@@ -2689,7 +2711,7 @@
         <v>15</v>
       </c>
       <c r="K54" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L54" s="16"/>
       <c r="M54" s="3"/>
@@ -2703,13 +2725,13 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="3"/>
       <c r="C55" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F55" s="11" t="n">
         <v>1</v>
@@ -2727,10 +2749,10 @@
         <v>30</v>
       </c>
       <c r="K55" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L55" s="32" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M55" s="3"/>
       <c r="N55" s="3"/>
@@ -2743,13 +2765,13 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="3"/>
       <c r="C56" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F56" s="11" t="n">
         <v>1</v>
@@ -2767,10 +2789,10 @@
         <v>90</v>
       </c>
       <c r="K56" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L56" s="32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M56" s="3"/>
       <c r="N56" s="3"/>
@@ -2783,13 +2805,13 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="3"/>
       <c r="C57" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F57" s="11" t="n">
         <v>1</v>
@@ -2807,10 +2829,10 @@
         <v>40</v>
       </c>
       <c r="K57" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L57" s="32" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
@@ -2846,7 +2868,7 @@
       </c>
       <c r="B59" s="3"/>
       <c r="C59" s="34" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D59" s="11"/>
       <c r="E59" s="11"/>
@@ -2868,13 +2890,13 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="3"/>
       <c r="C60" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F60" s="11" t="n">
         <v>1</v>
@@ -2892,10 +2914,10 @@
         <v>36</v>
       </c>
       <c r="K60" s="16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L60" s="32" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="M60" s="3"/>
       <c r="N60" s="3"/>
@@ -2908,13 +2930,13 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="3"/>
       <c r="C61" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F61" s="11" t="n">
         <v>1</v>
@@ -2932,10 +2954,10 @@
         <v>18</v>
       </c>
       <c r="K61" s="16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L61" s="32" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M61" s="3"/>
       <c r="N61" s="3"/>
@@ -2948,13 +2970,13 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="3"/>
       <c r="C62" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F62" s="11" t="n">
         <v>1</v>
@@ -2972,10 +2994,10 @@
         <v>18</v>
       </c>
       <c r="K62" s="16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L62" s="32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M62" s="3"/>
       <c r="N62" s="3"/>
@@ -2988,10 +3010,10 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="3"/>
       <c r="C63" s="11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E63" s="11"/>
       <c r="F63" s="11" t="n">
@@ -3010,10 +3032,10 @@
         <v>180</v>
       </c>
       <c r="K63" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L63" s="32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="M63" s="3"/>
       <c r="N63" s="3"/>
@@ -3042,7 +3064,7 @@
       </c>
       <c r="B65" s="3"/>
       <c r="C65" s="40" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J65" s="10"/>
       <c r="K65" s="3"/>
@@ -3058,13 +3080,13 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="3"/>
       <c r="C66" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F66" s="1" t="n">
         <v>1</v>
@@ -3082,10 +3104,10 @@
         <v>100</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L66" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M66" s="3"/>
       <c r="N66" s="3"/>
@@ -3098,13 +3120,13 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="3"/>
       <c r="C67" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F67" s="1" t="n">
         <v>1</v>
@@ -3122,10 +3144,10 @@
         <v>120</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L67" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M67" s="3"/>
       <c r="N67" s="3"/>
@@ -3138,13 +3160,13 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="3"/>
       <c r="C68" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F68" s="1" t="n">
         <v>1</v>
@@ -3162,10 +3184,10 @@
         <v>50</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L68" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M68" s="3"/>
       <c r="N68" s="3"/>
@@ -3178,13 +3200,13 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="3"/>
       <c r="C69" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>1</v>
@@ -3202,10 +3224,10 @@
         <v>50</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L69" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M69" s="3"/>
       <c r="N69" s="3"/>
@@ -3218,13 +3240,13 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="3"/>
       <c r="C70" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F70" s="1" t="n">
         <v>1</v>
@@ -3242,10 +3264,10 @@
         <v>105</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L70" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M70" s="3"/>
       <c r="N70" s="3"/>
@@ -3258,13 +3280,13 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="3"/>
       <c r="C71" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F71" s="1" t="n">
         <v>1</v>
@@ -3282,10 +3304,10 @@
         <v>40</v>
       </c>
       <c r="K71" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L71" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M71" s="3"/>
       <c r="N71" s="3"/>
@@ -3314,7 +3336,7 @@
       </c>
       <c r="B73" s="3"/>
       <c r="C73" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J73" s="10"/>
       <c r="K73" s="3"/>
@@ -3330,10 +3352,10 @@
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="3"/>
       <c r="C74" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>1</v>
@@ -3349,7 +3371,7 @@
       </c>
       <c r="J74" s="10"/>
       <c r="K74" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L74" s="3"/>
       <c r="M74" s="3"/>
@@ -3363,7 +3385,7 @@
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="3"/>
       <c r="E75" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F75" s="1" t="n">
         <v>1</v>
@@ -3379,7 +3401,7 @@
       </c>
       <c r="J75" s="10"/>
       <c r="K75" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L75" s="3"/>
       <c r="M75" s="3"/>
@@ -3393,13 +3415,13 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="3"/>
       <c r="C76" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="E76" s="9" t="s">
         <v>142</v>
-      </c>
-      <c r="D76" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="E76" s="9" t="s">
-        <v>140</v>
       </c>
       <c r="F76" s="1" t="n">
         <v>1</v>
@@ -3417,34 +3439,34 @@
         <v>25</v>
       </c>
       <c r="K76" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L76" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="N76" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="O76" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="P76" s="3"/>
       <c r="Q76" s="41" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R76" s="3"/>
       <c r="S76" s="3"/>
       <c r="T76" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="3"/>
       <c r="E77" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F77" s="1" t="n">
         <v>1</v>
@@ -3460,7 +3482,7 @@
       </c>
       <c r="J77" s="10"/>
       <c r="K77" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L77" s="3"/>
       <c r="M77" s="3"/>
@@ -3474,13 +3496,13 @@
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="3"/>
       <c r="C78" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>1</v>
@@ -3498,40 +3520,40 @@
         <v>20</v>
       </c>
       <c r="K78" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L78" s="33" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="N78" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="O78" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="P78" s="3"/>
       <c r="Q78" s="41" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="R78" s="3"/>
       <c r="S78" s="3"/>
       <c r="T78" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="3"/>
       <c r="C79" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>2</v>
@@ -3549,14 +3571,14 @@
         <v>60</v>
       </c>
       <c r="K79" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="L79" s="3"/>
       <c r="M79" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="N79" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="O79" s="3"/>
       <c r="P79" s="3"/>
@@ -3567,16 +3589,16 @@
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="3"/>
       <c r="D80" s="9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J80" s="10" t="n">
         <v>60</v>
       </c>
       <c r="K80" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L80" s="33" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="M80" s="3"/>
       <c r="N80" s="3"/>
@@ -3589,13 +3611,13 @@
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="3"/>
       <c r="C81" s="9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>1</v>
@@ -3613,23 +3635,23 @@
         <v>25</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L81" s="33" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="N81" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O81" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="P81" s="3"/>
       <c r="Q81" s="41" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="R81" s="3"/>
       <c r="S81" s="3"/>
@@ -3665,7 +3687,7 @@
       </c>
       <c r="B83" s="3"/>
       <c r="C83" s="9" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J83" s="10"/>
       <c r="K83" s="3"/>
@@ -3681,10 +3703,10 @@
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="3"/>
       <c r="C84" s="9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E84" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F84" s="1" t="n">
         <v>1</v>
@@ -3712,7 +3734,7 @@
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3"/>
       <c r="D85" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F85" s="1" t="n">
         <v>1</v>
@@ -3765,7 +3787,7 @@
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3"/>
       <c r="E87" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F87" s="1" t="n">
         <v>1</v>
@@ -3793,7 +3815,7 @@
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="3"/>
       <c r="C88" s="9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F88" s="1" t="n">
         <v>1</v>
@@ -3821,10 +3843,10 @@
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="3"/>
       <c r="C89" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F89" s="1" t="n">
         <v>2</v>
@@ -3852,13 +3874,13 @@
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="3"/>
       <c r="C90" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E90" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F90" s="1" t="n">
         <v>1</v>
@@ -3886,13 +3908,13 @@
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="3"/>
       <c r="C91" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D91" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F91" s="1" t="n">
         <v>1</v>
@@ -3920,7 +3942,7 @@
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="3"/>
       <c r="D92" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J92" s="10"/>
       <c r="K92" s="3"/>
@@ -3939,7 +3961,7 @@
       </c>
       <c r="B93" s="3"/>
       <c r="C93" s="9" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J93" s="10"/>
       <c r="K93" s="3"/>
@@ -3968,10 +3990,10 @@
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="3"/>
       <c r="C95" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F95" s="1" t="n">
         <v>1</v>
@@ -3999,10 +4021,10 @@
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="3"/>
       <c r="C96" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E96" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F96" s="1" t="n">
         <v>1</v>
@@ -4030,10 +4052,10 @@
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="3"/>
       <c r="C97" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F97" s="1" t="n">
         <v>1</v>
@@ -4086,10 +4108,10 @@
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="3"/>
       <c r="C99" s="9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F99" s="1" t="n">
         <v>1</v>
@@ -4122,46 +4144,50 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1" display="arnav.prasad.tech@gmail.com"/>
-    <hyperlink ref="Q3" r:id="rId2" display="arnav.prasad.tech@gmail.com"/>
-    <hyperlink ref="Q4" r:id="rId3" display="arnav.prasad.tech@gmail.com"/>
-    <hyperlink ref="Q5" r:id="rId4" display="arnav.prasad.tech@gmail.com"/>
-    <hyperlink ref="Q6" r:id="rId5" display="arnav.prasad.tech@gmail.com"/>
-    <hyperlink ref="L15" r:id="rId6" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EXHWOoyhaSxHm7Lao21I5xQBIQJnC9zkwJAsWTPrz0VqbQ?e=iPwYTM"/>
-    <hyperlink ref="L26" r:id="rId7" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EY7XfX1KNQlMkCTxXJQI0BABleLdKq1eLj2eJ2QNIOqH1A?e=GsPQog"/>
-    <hyperlink ref="L27" r:id="rId8" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EfGEwf925gBLsi9eaW-g3ykBCPS2_nS6iGvPHJ5mHA9sng?e=W93FeG"/>
-    <hyperlink ref="L28" r:id="rId9" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="L31" r:id="rId10" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=FfvEO4"/>
-    <hyperlink ref="L32" r:id="rId11" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/EQV193k-k_pNq0ihEG9vBHIBUbOPsCqlm1XRtDJ9Dwq6qw?e=qgBbbB"/>
-    <hyperlink ref="L33" r:id="rId12" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=yIhjgd"/>
-    <hyperlink ref="L38" r:id="rId13" display="Fluid Mechanics_Basement1.jpg"/>
-    <hyperlink ref="L39" r:id="rId14" display="App Mechanics_First Floor_Classroom.jpg"/>
-    <hyperlink ref="L42" r:id="rId15" display="App Mechanics_Classroom2.jpg"/>
-    <hyperlink ref="L43" r:id="rId16" display="App Mechanics Classroom1 (1).jpg"/>
-    <hyperlink ref="L45" r:id="rId17" display="App Mech Ground Floor Seminar Hall.jpg"/>
-    <hyperlink ref="L47" r:id="rId18" display="R22.jpg"/>
-    <hyperlink ref="L51" r:id="rId19" display="https://drive.google.com/file/d/11r8JUGcdvTO0ylOI_nn1YEYv9b4CKOKq/view?usp=sharing"/>
-    <hyperlink ref="L52" r:id="rId20" display="https://drive.google.com/file/d/1xfCJ7OavNoyQdfRC-VI19CAZpL4tOAEL/view?usp=sharing"/>
-    <hyperlink ref="L53" r:id="rId21" display="https://drive.google.com/file/d/1WSBvMorlthEbWyaCh8JdxRMas7G4kjVu/view?usp=sharing"/>
-    <hyperlink ref="L55" r:id="rId22" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
-    <hyperlink ref="L56" r:id="rId23" display="https://drive.google.com/file/d/1E-q97N6HQpt942F05ddKGT_D6nsHbDe_/view?usp=sharing"/>
-    <hyperlink ref="L57" r:id="rId24" display="https://drive.google.com/file/d/1orGoTWToL2cNbFSvNjVnGiJBTqj4-x7p/view?usp=sharing"/>
-    <hyperlink ref="L60" r:id="rId25" display="https://drive.google.com/file/d/1bJecDqhyMaVv0s9jZLgIDUpY1PGb-2qw/view?usp=sharing"/>
-    <hyperlink ref="L61" r:id="rId26" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
-    <hyperlink ref="L62" r:id="rId27" display="https://drive.google.com/file/d/1V56Qmp1d-mKg5U3SGllOvQp56yiec8hE/view?usp=sharing"/>
-    <hyperlink ref="L63" r:id="rId28" display="https://drive.google.com/file/d/1pcndMBRukVQKbKa81_jG_82Q2cZywHFu/view?usp=sharing"/>
-    <hyperlink ref="L66" r:id="rId29" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L67" r:id="rId30" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L68" r:id="rId31" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L69" r:id="rId32" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L70" r:id="rId33" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L71" r:id="rId34" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="L76" r:id="rId35" display="Env Classroom.jpeg"/>
-    <hyperlink ref="Q76" r:id="rId36" display="muk.civil@coep.ac.in"/>
-    <hyperlink ref="L78" r:id="rId37" display="CM Classroom.jpeg"/>
-    <hyperlink ref="Q78" r:id="rId38" display="gsv.civil@coeptech.ac.in"/>
-    <hyperlink ref="L80" r:id="rId39" display="R8.jpeg"/>
-    <hyperlink ref="L81" r:id="rId40" display="Geotech Classroom.jpeg"/>
-    <hyperlink ref="Q81" r:id="rId41" display="yak.civl@coeptech.ac.in"/>
+    <hyperlink ref="U2" r:id="rId2" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="Q3" r:id="rId3" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="U3" r:id="rId4" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="Q4" r:id="rId5" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="U4" r:id="rId6" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="Q5" r:id="rId7" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="U5" r:id="rId8" display="arnav.davpune@gmail.com"/>
+    <hyperlink ref="Q6" r:id="rId9" display="arnav.prasad.tech@gmail.com"/>
+    <hyperlink ref="L15" r:id="rId10" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EXHWOoyhaSxHm7Lao21I5xQBIQJnC9zkwJAsWTPrz0VqbQ?e=iPwYTM"/>
+    <hyperlink ref="L26" r:id="rId11" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EY7XfX1KNQlMkCTxXJQI0BABleLdKq1eLj2eJ2QNIOqH1A?e=GsPQog"/>
+    <hyperlink ref="L27" r:id="rId12" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EfGEwf925gBLsi9eaW-g3ykBCPS2_nS6iGvPHJ5mHA9sng?e=W93FeG"/>
+    <hyperlink ref="L28" r:id="rId13" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
+    <hyperlink ref="L31" r:id="rId14" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=FfvEO4"/>
+    <hyperlink ref="L32" r:id="rId15" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/EQV193k-k_pNq0ihEG9vBHIBUbOPsCqlm1XRtDJ9Dwq6qw?e=qgBbbB"/>
+    <hyperlink ref="L33" r:id="rId16" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=yIhjgd"/>
+    <hyperlink ref="L38" r:id="rId17" display="Fluid Mechanics_Basement1.jpg"/>
+    <hyperlink ref="L39" r:id="rId18" display="App Mechanics_First Floor_Classroom.jpg"/>
+    <hyperlink ref="L42" r:id="rId19" display="App Mechanics_Classroom2.jpg"/>
+    <hyperlink ref="L43" r:id="rId20" display="App Mechanics Classroom1 (1).jpg"/>
+    <hyperlink ref="L45" r:id="rId21" display="App Mech Ground Floor Seminar Hall.jpg"/>
+    <hyperlink ref="L47" r:id="rId22" display="R22.jpg"/>
+    <hyperlink ref="L51" r:id="rId23" display="https://drive.google.com/file/d/11r8JUGcdvTO0ylOI_nn1YEYv9b4CKOKq/view?usp=sharing"/>
+    <hyperlink ref="L52" r:id="rId24" display="https://drive.google.com/file/d/1xfCJ7OavNoyQdfRC-VI19CAZpL4tOAEL/view?usp=sharing"/>
+    <hyperlink ref="L53" r:id="rId25" display="https://drive.google.com/file/d/1WSBvMorlthEbWyaCh8JdxRMas7G4kjVu/view?usp=sharing"/>
+    <hyperlink ref="L55" r:id="rId26" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
+    <hyperlink ref="L56" r:id="rId27" display="https://drive.google.com/file/d/1E-q97N6HQpt942F05ddKGT_D6nsHbDe_/view?usp=sharing"/>
+    <hyperlink ref="L57" r:id="rId28" display="https://drive.google.com/file/d/1orGoTWToL2cNbFSvNjVnGiJBTqj4-x7p/view?usp=sharing"/>
+    <hyperlink ref="L60" r:id="rId29" display="https://drive.google.com/file/d/1bJecDqhyMaVv0s9jZLgIDUpY1PGb-2qw/view?usp=sharing"/>
+    <hyperlink ref="L61" r:id="rId30" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
+    <hyperlink ref="L62" r:id="rId31" display="https://drive.google.com/file/d/1V56Qmp1d-mKg5U3SGllOvQp56yiec8hE/view?usp=sharing"/>
+    <hyperlink ref="L63" r:id="rId32" display="https://drive.google.com/file/d/1pcndMBRukVQKbKa81_jG_82Q2cZywHFu/view?usp=sharing"/>
+    <hyperlink ref="L66" r:id="rId33" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L67" r:id="rId34" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L68" r:id="rId35" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L69" r:id="rId36" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L70" r:id="rId37" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L71" r:id="rId38" display="EED Classrooms_ 24 4 2025"/>
+    <hyperlink ref="L76" r:id="rId39" display="Env Classroom.jpeg"/>
+    <hyperlink ref="Q76" r:id="rId40" display="muk.civil@coep.ac.in"/>
+    <hyperlink ref="L78" r:id="rId41" display="CM Classroom.jpeg"/>
+    <hyperlink ref="Q78" r:id="rId42" display="gsv.civil@coeptech.ac.in"/>
+    <hyperlink ref="L80" r:id="rId43" display="R8.jpeg"/>
+    <hyperlink ref="L81" r:id="rId44" display="Geotech Classroom.jpeg"/>
+    <hyperlink ref="Q81" r:id="rId45" display="yak.civl@coeptech.ac.in"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4170,7 +4196,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId42"/>
+  <drawing r:id="rId46"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updated Venues Data file
</commit_message>
<xml_diff>
--- a/Data1.xlsx
+++ b/Data1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="191">
   <si>
     <t xml:space="preserve">Sr No</t>
   </si>
@@ -97,7 +97,7 @@
     <t xml:space="preserve">https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo</t>
   </si>
   <si>
-    <t xml:space="preserve">dean.engineering@coeptech.ac.in</t>
+    <t xml:space="preserve">hod.appsci@coeptech.ac.in</t>
   </si>
   <si>
     <t xml:space="preserve">Academic Complex 102</t>
@@ -175,6 +175,9 @@
     <t xml:space="preserve">2020-25507318</t>
   </si>
   <si>
+    <t xml:space="preserve">hod.extc@coeptech.ac.in</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mr. Shriraj Chavhan</t>
   </si>
   <si>
@@ -220,6 +223,9 @@
     <t xml:space="preserve">Instrumentation and Control</t>
   </si>
   <si>
+    <t xml:space="preserve">hod.instru@coeptech.ac.in</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/EQV193k-k_pNq0ihEG9vBHIBUbOPsCqlm1XRtDJ9Dwq6qw?e=qgBbbB</t>
   </si>
   <si>
@@ -247,6 +253,9 @@
     <t xml:space="preserve">Fluid Mechanics_Basement1.jpg</t>
   </si>
   <si>
+    <t xml:space="preserve">hod.mech@coeptech.ac.in</t>
+  </si>
+  <si>
     <t xml:space="preserve">First Floor</t>
   </si>
   <si>
@@ -361,9 +370,6 @@
     <t xml:space="preserve">Second Floor</t>
   </si>
   <si>
-    <t xml:space="preserve">ME-201 (New Building)</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://drive.google.com/file/d/1V56Qmp1d-mKg5U3SGllOvQp56yiec8hE/view?usp=sharing</t>
   </si>
   <si>
@@ -385,6 +391,9 @@
     <t xml:space="preserve">EED Classrooms_ 24 4 2025</t>
   </si>
   <si>
+    <t xml:space="preserve">hod.elec@coeptech.ac.in</t>
+  </si>
+  <si>
     <t xml:space="preserve">Electrical Engg Dept</t>
   </si>
   <si>
@@ -433,6 +442,9 @@
     <t xml:space="preserve">Projector , Podium</t>
   </si>
   <si>
+    <t xml:space="preserve">hod.civil@coeptech.ac.in</t>
+  </si>
+  <si>
     <t xml:space="preserve">1st Floor (Environment Lab)</t>
   </si>
   <si>
@@ -515,6 +527,9 @@
   </si>
   <si>
     <t xml:space="preserve">Production Class Room 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hod.prod@coeptech.ac.in</t>
   </si>
   <si>
     <r>
@@ -566,6 +581,9 @@
   </si>
   <si>
     <t xml:space="preserve">MM-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hod.meta@coeptech.ac.in</t>
   </si>
   <si>
     <t xml:space="preserve">MM-101</t>
@@ -849,7 +867,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -991,6 +1009,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1874,14 +1896,14 @@
       <c r="P10" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="Q10" s="4" t="s">
-        <v>25</v>
+      <c r="Q10" s="29" t="s">
+        <v>51</v>
       </c>
       <c r="R10" s="29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S10" s="29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="T10" s="29" t="s">
         <v>36</v>
@@ -1894,16 +1916,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F11" s="13" t="n">
         <v>1</v>
@@ -1926,8 +1948,8 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
-      <c r="Q11" s="4" t="s">
-        <v>25</v>
+      <c r="Q11" s="29" t="s">
+        <v>51</v>
       </c>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
@@ -1937,16 +1959,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F12" s="13" t="n">
         <v>1</v>
@@ -1969,8 +1991,8 @@
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
-      <c r="Q12" s="4" t="s">
-        <v>25</v>
+      <c r="Q12" s="29" t="s">
+        <v>51</v>
       </c>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
@@ -1980,16 +2002,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F13" s="13" t="n">
         <v>1</v>
@@ -2012,8 +2034,8 @@
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
-      <c r="Q13" s="4" t="s">
-        <v>25</v>
+      <c r="Q13" s="29" t="s">
+        <v>51</v>
       </c>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
@@ -2023,13 +2045,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>45</v>
@@ -2055,24 +2077,24 @@
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
-      <c r="Q14" s="4" t="s">
-        <v>25</v>
+      <c r="Q14" s="29" t="s">
+        <v>51</v>
       </c>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="36" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E15" s="33" t="s">
         <v>45</v>
@@ -2092,22 +2114,31 @@
       <c r="J15" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="Q15" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="K15" s="35"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35"/>
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="35"/>
+      <c r="Q15" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="R15" s="35"/>
+      <c r="S15" s="35"/>
+      <c r="T15" s="35"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="36" t="s">
-        <v>60</v>
+      <c r="B16" s="37" t="s">
+        <v>61</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>45</v>
@@ -2128,23 +2159,23 @@
         <v>40</v>
       </c>
       <c r="K16" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M16" s="19" t="s">
         <v>33</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O16" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P16" s="18"/>
-      <c r="Q16" s="4" t="s">
-        <v>25</v>
+      <c r="Q16" s="18" t="s">
+        <v>67</v>
       </c>
       <c r="R16" s="18"/>
       <c r="S16" s="18"/>
@@ -2154,11 +2185,11 @@
       <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="36" t="s">
-        <v>60</v>
+      <c r="B17" s="37" t="s">
+        <v>61</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>23</v>
@@ -2184,21 +2215,21 @@
       <c r="K17" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L17" s="37" t="s">
-        <v>66</v>
+      <c r="L17" s="38" t="s">
+        <v>68</v>
       </c>
       <c r="M17" s="19" t="s">
         <v>33</v>
       </c>
       <c r="N17" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="O17" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18" t="s">
         <v>67</v>
-      </c>
-      <c r="O17" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="P17" s="18"/>
-      <c r="Q17" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="R17" s="18"/>
       <c r="S17" s="18"/>
@@ -2208,14 +2239,14 @@
       <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="36" t="s">
-        <v>60</v>
+      <c r="B18" s="37" t="s">
+        <v>61</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E18" s="13" t="s">
         <v>45</v>
@@ -2239,40 +2270,40 @@
         <v>46</v>
       </c>
       <c r="L18" s="19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="M18" s="19" t="s">
         <v>33</v>
       </c>
       <c r="N18" s="18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O18" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P18" s="18"/>
-      <c r="Q18" s="4" t="s">
-        <v>25</v>
+      <c r="Q18" s="18" t="s">
+        <v>67</v>
       </c>
       <c r="R18" s="18"/>
       <c r="S18" s="18"/>
       <c r="T18" s="18"/>
     </row>
-    <row r="19" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" s="36" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="38" t="s">
-        <v>71</v>
+      <c r="B19" s="39" t="s">
+        <v>73</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F19" s="33" t="n">
         <v>1</v>
@@ -2290,25 +2321,32 @@
         <v>30</v>
       </c>
       <c r="K19" s="33"/>
-      <c r="L19" s="39" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q19" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="L19" s="40" t="s">
+        <v>76</v>
+      </c>
+      <c r="M19" s="35"/>
+      <c r="N19" s="35"/>
+      <c r="O19" s="35"/>
+      <c r="P19" s="35"/>
+      <c r="Q19" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="R19" s="35"/>
+      <c r="S19" s="35"/>
+      <c r="T19" s="35"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>23</v>
@@ -2329,17 +2367,17 @@
         <v>30</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L20" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="L20" s="41" t="s">
+        <v>81</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
-      <c r="Q20" s="4" t="s">
-        <v>25</v>
+      <c r="Q20" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
@@ -2349,13 +2387,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>23</v>
@@ -2376,15 +2414,15 @@
         <v>30</v>
       </c>
       <c r="K21" s="18"/>
-      <c r="L21" s="40" t="s">
-        <v>80</v>
+      <c r="L21" s="41" t="s">
+        <v>83</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
-      <c r="Q21" s="4" t="s">
-        <v>25</v>
+      <c r="Q21" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
@@ -2394,13 +2432,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>23</v>
@@ -2421,15 +2459,15 @@
         <v>30</v>
       </c>
       <c r="K22" s="18"/>
-      <c r="L22" s="40" t="s">
-        <v>82</v>
+      <c r="L22" s="41" t="s">
+        <v>85</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
-      <c r="Q22" s="4" t="s">
-        <v>25</v>
+      <c r="Q22" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
@@ -2439,13 +2477,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>44</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>45</v>
@@ -2466,17 +2504,17 @@
         <v>40</v>
       </c>
       <c r="K23" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L23" s="40" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="L23" s="41" t="s">
+        <v>87</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
       <c r="P23" s="4"/>
-      <c r="Q23" s="4" t="s">
-        <v>25</v>
+      <c r="Q23" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
@@ -2486,13 +2524,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E24" s="13" t="s">
         <v>23</v>
@@ -2513,17 +2551,17 @@
         <v>80</v>
       </c>
       <c r="K24" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L24" s="40" t="s">
-        <v>86</v>
+        <v>80</v>
+      </c>
+      <c r="L24" s="41" t="s">
+        <v>89</v>
       </c>
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
-      <c r="Q24" s="4" t="s">
-        <v>25</v>
+      <c r="Q24" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
@@ -2532,17 +2570,17 @@
       <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="41" t="s">
-        <v>87</v>
+      <c r="B25" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F25" s="13" t="n">
         <v>1</v>
@@ -2550,21 +2588,21 @@
       <c r="G25" s="13"/>
       <c r="H25" s="13"/>
       <c r="I25" s="13"/>
-      <c r="J25" s="42" t="n">
+      <c r="J25" s="43" t="n">
         <v>90</v>
       </c>
       <c r="K25" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="L25" s="43" t="s">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="L25" s="44" t="s">
+        <v>94</v>
       </c>
       <c r="M25" s="4"/>
       <c r="N25" s="4"/>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
-      <c r="Q25" s="4" t="s">
-        <v>25</v>
+      <c r="Q25" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
@@ -2573,17 +2611,17 @@
       <c r="A26" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="41" t="s">
-        <v>87</v>
+      <c r="B26" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D26" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>92</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>89</v>
       </c>
       <c r="F26" s="13" t="n">
         <v>1</v>
@@ -2591,21 +2629,21 @@
       <c r="G26" s="13"/>
       <c r="H26" s="13"/>
       <c r="I26" s="13"/>
-      <c r="J26" s="42" t="n">
+      <c r="J26" s="43" t="n">
         <v>120</v>
       </c>
       <c r="K26" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="L26" s="43" t="s">
         <v>93</v>
+      </c>
+      <c r="L26" s="44" t="s">
+        <v>96</v>
       </c>
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
-      <c r="Q26" s="4" t="s">
-        <v>25</v>
+      <c r="Q26" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
@@ -2614,17 +2652,17 @@
       <c r="A27" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="41" t="s">
-        <v>87</v>
+      <c r="B27" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F27" s="13" t="n">
         <v>1</v>
@@ -2632,21 +2670,21 @@
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
       <c r="I27" s="13"/>
-      <c r="J27" s="42" t="n">
+      <c r="J27" s="43" t="n">
         <v>120</v>
       </c>
       <c r="K27" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="L27" s="43" t="s">
-        <v>95</v>
+        <v>93</v>
+      </c>
+      <c r="L27" s="44" t="s">
+        <v>98</v>
       </c>
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
-      <c r="Q27" s="4" t="s">
-        <v>25</v>
+      <c r="Q27" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
@@ -2655,17 +2693,17 @@
       <c r="A28" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="41" t="s">
-        <v>87</v>
+      <c r="B28" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F28" s="13" t="n">
         <v>1</v>
@@ -2673,19 +2711,19 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
-      <c r="J28" s="42" t="n">
+      <c r="J28" s="43" t="n">
         <v>15</v>
       </c>
       <c r="K28" s="18" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="L28" s="18"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
-      <c r="Q28" s="4" t="s">
-        <v>25</v>
+      <c r="Q28" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
@@ -2694,45 +2732,45 @@
       <c r="A29" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="41" t="s">
-        <v>87</v>
+      <c r="B29" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F29" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="44" t="n">
+      <c r="G29" s="45" t="n">
         <v>30</v>
       </c>
-      <c r="H29" s="45" t="n">
+      <c r="H29" s="46" t="n">
         <v>20.8</v>
       </c>
-      <c r="I29" s="45" t="n">
+      <c r="I29" s="46" t="n">
         <v>624</v>
       </c>
-      <c r="J29" s="42" t="n">
+      <c r="J29" s="43" t="n">
         <v>30</v>
       </c>
       <c r="K29" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="L29" s="43" t="s">
         <v>100</v>
+      </c>
+      <c r="L29" s="44" t="s">
+        <v>103</v>
       </c>
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
-      <c r="Q29" s="4" t="s">
-        <v>25</v>
+      <c r="Q29" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
@@ -2741,45 +2779,45 @@
       <c r="A30" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="41" t="s">
-        <v>87</v>
+      <c r="B30" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F30" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="44" t="n">
+      <c r="G30" s="45" t="n">
         <v>48</v>
       </c>
-      <c r="H30" s="45" t="n">
+      <c r="H30" s="46" t="n">
         <v>24.8</v>
       </c>
-      <c r="I30" s="45" t="n">
+      <c r="I30" s="46" t="n">
         <v>1190.4</v>
       </c>
-      <c r="J30" s="42" t="n">
+      <c r="J30" s="43" t="n">
         <v>90</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="L30" s="43" t="s">
-        <v>103</v>
+        <v>93</v>
+      </c>
+      <c r="L30" s="44" t="s">
+        <v>106</v>
       </c>
       <c r="M30" s="4"/>
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
-      <c r="Q30" s="4" t="s">
-        <v>25</v>
+      <c r="Q30" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
@@ -2788,45 +2826,45 @@
       <c r="A31" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="41" t="s">
-        <v>87</v>
+      <c r="B31" s="42" t="s">
+        <v>90</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>29</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F31" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="46" t="n">
+      <c r="G31" s="47" t="n">
         <v>29.1</v>
       </c>
-      <c r="H31" s="47" t="n">
+      <c r="H31" s="48" t="n">
         <v>21.5</v>
       </c>
-      <c r="I31" s="47" t="n">
+      <c r="I31" s="48" t="n">
         <v>625.65</v>
       </c>
-      <c r="J31" s="42" t="n">
+      <c r="J31" s="43" t="n">
         <v>40</v>
       </c>
       <c r="K31" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="L31" s="43" t="s">
-        <v>105</v>
+        <v>100</v>
+      </c>
+      <c r="L31" s="44" t="s">
+        <v>108</v>
       </c>
       <c r="M31" s="4"/>
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
-      <c r="Q31" s="4" t="s">
-        <v>25</v>
+      <c r="Q31" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
@@ -2835,45 +2873,45 @@
       <c r="A32" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="48" t="s">
-        <v>106</v>
+      <c r="B32" s="49" t="s">
+        <v>109</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F32" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="44" t="n">
+      <c r="G32" s="45" t="n">
         <v>44.8</v>
       </c>
-      <c r="H32" s="45" t="n">
+      <c r="H32" s="46" t="n">
         <v>24.11</v>
       </c>
-      <c r="I32" s="45" t="n">
+      <c r="I32" s="46" t="n">
         <v>1080.128</v>
       </c>
-      <c r="J32" s="42" t="n">
+      <c r="J32" s="43" t="n">
         <v>36</v>
       </c>
       <c r="K32" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="L32" s="43" t="s">
-        <v>110</v>
+        <v>112</v>
+      </c>
+      <c r="L32" s="44" t="s">
+        <v>113</v>
       </c>
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
-      <c r="Q32" s="4" t="s">
-        <v>25</v>
+      <c r="Q32" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
@@ -2882,45 +2920,45 @@
       <c r="A33" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="48" t="s">
-        <v>106</v>
+      <c r="B33" s="49" t="s">
+        <v>109</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D33" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E33" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E33" s="13" t="s">
-        <v>108</v>
-      </c>
       <c r="F33" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="46" t="n">
+      <c r="G33" s="47" t="n">
         <v>25.01</v>
       </c>
-      <c r="H33" s="47" t="n">
+      <c r="H33" s="48" t="n">
         <v>18.8</v>
       </c>
-      <c r="I33" s="47" t="n">
+      <c r="I33" s="48" t="n">
         <v>470.188</v>
       </c>
-      <c r="J33" s="42" t="n">
+      <c r="J33" s="43" t="n">
         <v>18</v>
       </c>
       <c r="K33" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="L33" s="43" t="s">
-        <v>100</v>
+        <v>112</v>
+      </c>
+      <c r="L33" s="44" t="s">
+        <v>103</v>
       </c>
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
-      <c r="Q33" s="4" t="s">
-        <v>25</v>
+      <c r="Q33" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
@@ -2929,103 +2967,110 @@
       <c r="A34" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="48" t="s">
-        <v>106</v>
+      <c r="B34" s="49" t="s">
+        <v>109</v>
       </c>
       <c r="C34" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="47" t="n">
+        <v>25.01</v>
+      </c>
+      <c r="H34" s="48" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="I34" s="48" t="n">
+        <v>470.188</v>
+      </c>
+      <c r="J34" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="K34" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="D34" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="F34" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="46" t="n">
-        <v>25.01</v>
-      </c>
-      <c r="H34" s="47" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="I34" s="47" t="n">
-        <v>470.188</v>
-      </c>
-      <c r="J34" s="42" t="n">
-        <v>18</v>
-      </c>
-      <c r="K34" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="L34" s="43" t="s">
-        <v>114</v>
+      <c r="L34" s="44" t="s">
+        <v>116</v>
       </c>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
-      <c r="Q34" s="4" t="s">
-        <v>25</v>
+      <c r="Q34" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" s="36" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="31" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="49" t="s">
-        <v>106</v>
+      <c r="B35" s="50" t="s">
+        <v>109</v>
       </c>
       <c r="C35" s="32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E35" s="33"/>
       <c r="F35" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="G35" s="50" t="n">
+      <c r="G35" s="51" t="n">
         <v>117</v>
       </c>
-      <c r="H35" s="51" t="n">
+      <c r="H35" s="52" t="n">
         <v>41</v>
       </c>
-      <c r="I35" s="51" t="n">
+      <c r="I35" s="52" t="n">
         <v>4797</v>
       </c>
-      <c r="J35" s="52" t="n">
+      <c r="J35" s="53" t="n">
         <v>180</v>
       </c>
       <c r="K35" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="L35" s="54" t="s">
+        <v>118</v>
+      </c>
+      <c r="M35" s="35"/>
+      <c r="N35" s="35"/>
+      <c r="O35" s="35"/>
+      <c r="P35" s="35"/>
+      <c r="Q35" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="L35" s="53" t="s">
-        <v>116</v>
-      </c>
-      <c r="Q35" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="R35" s="35"/>
+      <c r="S35" s="35"/>
+      <c r="T35" s="35"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F36" s="13" t="n">
         <v>1</v>
@@ -3043,17 +3088,17 @@
         <v>100</v>
       </c>
       <c r="K36" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="L36" s="40" t="s">
-        <v>120</v>
+        <v>121</v>
+      </c>
+      <c r="L36" s="41" t="s">
+        <v>122</v>
       </c>
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
       <c r="Q36" s="4" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
@@ -3062,17 +3107,17 @@
       <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="54" t="s">
-        <v>121</v>
+      <c r="B37" s="55" t="s">
+        <v>124</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F37" s="13" t="n">
         <v>1</v>
@@ -3090,17 +3135,17 @@
         <v>120</v>
       </c>
       <c r="K37" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L37" s="40" t="s">
-        <v>120</v>
+        <v>80</v>
+      </c>
+      <c r="L37" s="41" t="s">
+        <v>122</v>
       </c>
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
       <c r="P37" s="4"/>
       <c r="Q37" s="4" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="R37" s="4"/>
       <c r="S37" s="4"/>
@@ -3109,17 +3154,17 @@
       <c r="A38" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="54" t="s">
-        <v>121</v>
+      <c r="B38" s="55" t="s">
+        <v>124</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F38" s="13" t="n">
         <v>1</v>
@@ -3137,17 +3182,17 @@
         <v>50</v>
       </c>
       <c r="K38" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L38" s="40" t="s">
-        <v>120</v>
+        <v>80</v>
+      </c>
+      <c r="L38" s="41" t="s">
+        <v>122</v>
       </c>
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
       <c r="P38" s="4"/>
       <c r="Q38" s="4" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
@@ -3156,17 +3201,17 @@
       <c r="A39" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="54" t="s">
-        <v>121</v>
+      <c r="B39" s="55" t="s">
+        <v>124</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F39" s="13" t="n">
         <v>1</v>
@@ -3184,17 +3229,17 @@
         <v>50</v>
       </c>
       <c r="K39" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L39" s="40" t="s">
-        <v>120</v>
+        <v>80</v>
+      </c>
+      <c r="L39" s="41" t="s">
+        <v>122</v>
       </c>
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
       <c r="Q39" s="4" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
@@ -3203,17 +3248,17 @@
       <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="54" t="s">
-        <v>121</v>
+      <c r="B40" s="55" t="s">
+        <v>124</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F40" s="13" t="n">
         <v>1</v>
@@ -3231,36 +3276,36 @@
         <v>105</v>
       </c>
       <c r="K40" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L40" s="40" t="s">
-        <v>120</v>
+        <v>80</v>
+      </c>
+      <c r="L40" s="41" t="s">
+        <v>122</v>
       </c>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
       <c r="Q40" s="4" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" s="36" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="31" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="55" t="s">
-        <v>121</v>
+      <c r="B41" s="56" t="s">
+        <v>124</v>
       </c>
       <c r="C41" s="32" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F41" s="33" t="n">
         <v>1</v>
@@ -3278,30 +3323,37 @@
         <v>40</v>
       </c>
       <c r="K41" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="L41" s="39" t="s">
-        <v>120</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="L41" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="M41" s="35"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
+      <c r="P41" s="35"/>
       <c r="Q41" s="4" t="s">
-        <v>25</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="R41" s="35"/>
+      <c r="S41" s="35"/>
+      <c r="T41" s="35"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="56" t="s">
-        <v>132</v>
+      <c r="B42" s="57" t="s">
+        <v>135</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F42" s="13" t="n">
         <v>1</v>
@@ -3317,7 +3369,7 @@
       </c>
       <c r="J42" s="14"/>
       <c r="K42" s="18" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="L42" s="4"/>
       <c r="M42" s="4"/>
@@ -3325,7 +3377,7 @@
       <c r="O42" s="4"/>
       <c r="P42" s="4"/>
       <c r="Q42" s="4" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
@@ -3334,17 +3386,17 @@
       <c r="A43" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="56" t="s">
-        <v>132</v>
+      <c r="B43" s="57" t="s">
+        <v>135</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D43" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E43" s="13" t="s">
         <v>138</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>135</v>
       </c>
       <c r="F43" s="13" t="n">
         <v>1</v>
@@ -3362,45 +3414,45 @@
         <v>25</v>
       </c>
       <c r="K43" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="L43" s="40" t="s">
-        <v>139</v>
+        <v>80</v>
+      </c>
+      <c r="L43" s="41" t="s">
+        <v>143</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="N43" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="O43" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="P43" s="4"/>
       <c r="Q43" s="4" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="R43" s="4"/>
       <c r="S43" s="4"/>
       <c r="T43" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="56" t="s">
-        <v>132</v>
+      <c r="B44" s="57" t="s">
+        <v>135</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F44" s="13" t="n">
         <v>1</v>
@@ -3418,45 +3470,45 @@
         <v>20</v>
       </c>
       <c r="K44" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="L44" s="40" t="s">
-        <v>147</v>
+        <v>150</v>
+      </c>
+      <c r="L44" s="41" t="s">
+        <v>151</v>
       </c>
       <c r="M44" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N44" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="O44" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="P44" s="4"/>
       <c r="Q44" s="4" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="R44" s="4"/>
       <c r="S44" s="4"/>
       <c r="T44" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="56" t="s">
-        <v>132</v>
+      <c r="B45" s="57" t="s">
+        <v>135</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F45" s="13" t="n">
         <v>2</v>
@@ -3474,19 +3526,19 @@
         <v>60</v>
       </c>
       <c r="K45" s="18" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="L45" s="4"/>
       <c r="M45" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N45" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="O45" s="4"/>
       <c r="P45" s="4"/>
       <c r="Q45" s="4" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
@@ -3495,14 +3547,14 @@
       <c r="A46" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="56" t="s">
-        <v>132</v>
+      <c r="B46" s="57" t="s">
+        <v>135</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E46" s="13"/>
       <c r="F46" s="13"/>
@@ -3513,36 +3565,36 @@
         <v>60</v>
       </c>
       <c r="K46" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="L46" s="40" t="s">
-        <v>155</v>
+        <v>158</v>
+      </c>
+      <c r="L46" s="41" t="s">
+        <v>159</v>
       </c>
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4"/>
       <c r="P46" s="4"/>
       <c r="Q46" s="4" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" s="36" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="31" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="57" t="s">
-        <v>132</v>
+      <c r="B47" s="58" t="s">
+        <v>135</v>
       </c>
       <c r="C47" s="32" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E47" s="33" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="F47" s="33" t="n">
         <v>1</v>
@@ -3560,39 +3612,43 @@
         <v>25</v>
       </c>
       <c r="K47" s="33" t="s">
-        <v>146</v>
-      </c>
-      <c r="L47" s="39" t="s">
-        <v>159</v>
+        <v>150</v>
+      </c>
+      <c r="L47" s="40" t="s">
+        <v>163</v>
       </c>
       <c r="M47" s="35" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N47" s="35" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="O47" s="35" t="s">
-        <v>161</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="P47" s="35"/>
       <c r="Q47" s="4" t="s">
-        <v>25</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="R47" s="35"/>
+      <c r="S47" s="35"/>
+      <c r="T47" s="35"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F48" s="13" t="n">
         <v>1</v>
@@ -3609,14 +3665,14 @@
       <c r="J48" s="14"/>
       <c r="K48" s="17"/>
       <c r="L48" s="18" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4"/>
       <c r="P48" s="4"/>
       <c r="Q48" s="4" t="s">
-        <v>25</v>
+        <v>169</v>
       </c>
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
@@ -3626,16 +3682,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F49" s="13" t="n">
         <v>1</v>
@@ -3657,7 +3713,7 @@
       <c r="O49" s="4"/>
       <c r="P49" s="4"/>
       <c r="Q49" s="4" t="s">
-        <v>25</v>
+        <v>169</v>
       </c>
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
@@ -3667,16 +3723,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F50" s="13" t="n">
         <v>1</v>
@@ -3698,7 +3754,7 @@
       <c r="O50" s="4"/>
       <c r="P50" s="4"/>
       <c r="Q50" s="4" t="s">
-        <v>25</v>
+        <v>169</v>
       </c>
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
@@ -3708,16 +3764,16 @@
         <v>51</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F51" s="13" t="n">
         <v>1</v>
@@ -3734,33 +3790,33 @@
       <c r="J51" s="14"/>
       <c r="K51" s="17"/>
       <c r="L51" s="18" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="M51" s="4"/>
       <c r="N51" s="4"/>
       <c r="O51" s="4"/>
       <c r="P51" s="4"/>
       <c r="Q51" s="4" t="s">
-        <v>25</v>
+        <v>169</v>
       </c>
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" s="35" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" s="36" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="31" t="n">
         <v>52</v>
       </c>
-      <c r="B52" s="38" t="s">
-        <v>162</v>
+      <c r="B52" s="39" t="s">
+        <v>166</v>
       </c>
       <c r="C52" s="32" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D52" s="33" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E52" s="33" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F52" s="33" t="n">
         <v>1</v>
@@ -3775,24 +3831,31 @@
         <v>32.22</v>
       </c>
       <c r="J52" s="34"/>
-      <c r="K52" s="58"/>
+      <c r="K52" s="59"/>
       <c r="L52" s="33"/>
+      <c r="M52" s="35"/>
+      <c r="N52" s="35"/>
+      <c r="O52" s="35"/>
+      <c r="P52" s="35"/>
       <c r="Q52" s="4" t="s">
-        <v>25</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="R52" s="35"/>
+      <c r="S52" s="35"/>
+      <c r="T52" s="35"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="n">
         <v>53</v>
       </c>
-      <c r="B53" s="54" t="s">
-        <v>170</v>
+      <c r="B53" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="E53" s="13" t="s">
         <v>23</v>
@@ -3819,7 +3882,7 @@
       <c r="O53" s="4"/>
       <c r="P53" s="4"/>
       <c r="Q53" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
@@ -3828,14 +3891,14 @@
       <c r="A54" s="1" t="n">
         <v>54</v>
       </c>
-      <c r="B54" s="54" t="s">
-        <v>170</v>
+      <c r="B54" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E54" s="13" t="s">
         <v>23</v>
@@ -3862,7 +3925,7 @@
       <c r="O54" s="4"/>
       <c r="P54" s="4"/>
       <c r="Q54" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
@@ -3871,14 +3934,14 @@
       <c r="A55" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="B55" s="54" t="s">
-        <v>170</v>
+      <c r="B55" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="E55" s="13" t="s">
         <v>23</v>
@@ -3905,7 +3968,7 @@
       <c r="O55" s="4"/>
       <c r="P55" s="4"/>
       <c r="Q55" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
@@ -3914,14 +3977,14 @@
       <c r="A56" s="1" t="n">
         <v>56</v>
       </c>
-      <c r="B56" s="54" t="s">
-        <v>170</v>
+      <c r="B56" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E56" s="13"/>
       <c r="F56" s="13" t="n">
@@ -3946,7 +4009,7 @@
       <c r="O56" s="4"/>
       <c r="P56" s="4"/>
       <c r="Q56" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
@@ -3955,17 +4018,17 @@
       <c r="A57" s="1" t="n">
         <v>57</v>
       </c>
-      <c r="B57" s="54" t="s">
-        <v>170</v>
+      <c r="B57" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F57" s="13" t="n">
         <v>1</v>
@@ -3989,7 +4052,7 @@
       <c r="O57" s="4"/>
       <c r="P57" s="4"/>
       <c r="Q57" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
@@ -3998,14 +4061,14 @@
       <c r="A58" s="1" t="n">
         <v>58</v>
       </c>
-      <c r="B58" s="54" t="s">
-        <v>170</v>
+      <c r="B58" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E58" s="13"/>
       <c r="F58" s="13"/>
@@ -4022,7 +4085,7 @@
       <c r="O58" s="4"/>
       <c r="P58" s="4"/>
       <c r="Q58" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
@@ -4031,14 +4094,14 @@
       <c r="A59" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="B59" s="54" t="s">
-        <v>170</v>
+      <c r="B59" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="E59" s="13"/>
       <c r="F59" s="13"/>
@@ -4055,7 +4118,7 @@
       <c r="O59" s="4"/>
       <c r="P59" s="4"/>
       <c r="Q59" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
@@ -4064,14 +4127,14 @@
       <c r="A60" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="B60" s="54" t="s">
-        <v>170</v>
+      <c r="B60" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E60" s="13"/>
       <c r="F60" s="13"/>
@@ -4088,7 +4151,7 @@
       <c r="O60" s="4"/>
       <c r="P60" s="4"/>
       <c r="Q60" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
@@ -4097,14 +4160,14 @@
       <c r="A61" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="B61" s="54" t="s">
-        <v>170</v>
-      </c>
-      <c r="C61" s="59" t="s">
-        <v>57</v>
+      <c r="B61" s="55" t="s">
+        <v>175</v>
+      </c>
+      <c r="C61" s="60" t="s">
+        <v>58</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E61" s="13"/>
       <c r="F61" s="13"/>
@@ -4121,7 +4184,7 @@
       <c r="O61" s="4"/>
       <c r="P61" s="4"/>
       <c r="Q61" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
@@ -4130,14 +4193,14 @@
       <c r="A62" s="1" t="n">
         <v>62</v>
       </c>
-      <c r="B62" s="54" t="s">
-        <v>170</v>
+      <c r="B62" s="55" t="s">
+        <v>175</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="E62" s="13"/>
       <c r="F62" s="13"/>
@@ -4154,13 +4217,13 @@
       <c r="O62" s="4"/>
       <c r="P62" s="4"/>
       <c r="Q62" s="4" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="60"/>
+      <c r="B63" s="61"/>
     </row>
     <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -4212,104 +4275,104 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="L2" r:id="rId1" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="Q2" r:id="rId2" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q2" r:id="rId2" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L3" r:id="rId3" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="Q3" r:id="rId4" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q3" r:id="rId4" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L4" r:id="rId5" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="Q4" r:id="rId6" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q4" r:id="rId6" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L5" r:id="rId7" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="Q5" r:id="rId8" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q5" r:id="rId8" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L6" r:id="rId9" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EY7XfX1KNQlMkCTxXJQI0BABleLdKq1eLj2eJ2QNIOqH1A?e=GsPQog"/>
-    <hyperlink ref="Q6" r:id="rId10" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q6" r:id="rId10" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L7" r:id="rId11" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EfGEwf925gBLsi9eaW-g3ykBCPS2_nS6iGvPHJ5mHA9sng?e=W93FeG"/>
-    <hyperlink ref="Q7" r:id="rId12" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q7" r:id="rId12" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L8" r:id="rId13" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="Q8" r:id="rId14" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q8" r:id="rId14" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L9" r:id="rId15" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/ERduddtqsJtIm4vagtvySXMB-Qy2JgeP6JgyjARhwvcrfA?e=2yJlmo"/>
-    <hyperlink ref="Q9" r:id="rId16" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q9" r:id="rId16" display="hod.appsci@coeptech.ac.in"/>
     <hyperlink ref="L10" r:id="rId17" display="https://coepac-my.sharepoint.com/:i:/g/personal/ksp_comp_coeptech_ac_in/EXHWOoyhaSxHm7Lao21I5xQBIQJnC9zkwJAsWTPrz0VqbQ?e=iPwYTM"/>
-    <hyperlink ref="Q10" r:id="rId18" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q11" r:id="rId19" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q12" r:id="rId20" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q13" r:id="rId21" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q14" r:id="rId22" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q15" r:id="rId23" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q10" r:id="rId18" display="hod.extc@coeptech.ac.in"/>
+    <hyperlink ref="Q11" r:id="rId19" display="hod.extc@coeptech.ac.in"/>
+    <hyperlink ref="Q12" r:id="rId20" display="hod.extc@coeptech.ac.in"/>
+    <hyperlink ref="Q13" r:id="rId21" display="hod.extc@coeptech.ac.in"/>
+    <hyperlink ref="Q14" r:id="rId22" display="hod.extc@coeptech.ac.in"/>
+    <hyperlink ref="Q15" r:id="rId23" display="hod.extc@coeptech.ac.in"/>
     <hyperlink ref="L16" r:id="rId24" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=FfvEO4"/>
-    <hyperlink ref="Q16" r:id="rId25" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q16" r:id="rId25" display="hod.instru@coeptech.ac.in"/>
     <hyperlink ref="L17" r:id="rId26" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/EQV193k-k_pNq0ihEG9vBHIBUbOPsCqlm1XRtDJ9Dwq6qw?e=qgBbbB"/>
-    <hyperlink ref="Q17" r:id="rId27" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q17" r:id="rId27" display="hod.instru@coeptech.ac.in"/>
     <hyperlink ref="L18" r:id="rId28" display="https://coepac-my.sharepoint.com/:i:/g/personal/kab_instru_coeptech_ac_in/Edav63Kjl2BLiMK7zwACu1gBt1v2VpqIYJvCvYyvpEESGg?e=yIhjgd"/>
-    <hyperlink ref="Q18" r:id="rId29" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q18" r:id="rId29" display="hod.instru@coeptech.ac.in"/>
     <hyperlink ref="L19" r:id="rId30" display="Fluid Mechanics_Basement1.jpg"/>
-    <hyperlink ref="Q19" r:id="rId31" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q19" r:id="rId31" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L20" r:id="rId32" display="App Mechanics_First Floor_Classroom.jpg"/>
-    <hyperlink ref="Q20" r:id="rId33" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q20" r:id="rId33" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L21" r:id="rId34" display="App Mechanics_Classroom2.jpg"/>
-    <hyperlink ref="Q21" r:id="rId35" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q21" r:id="rId35" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L22" r:id="rId36" display="App Mechanics Classroom1 (1).jpg"/>
-    <hyperlink ref="Q22" r:id="rId37" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q22" r:id="rId37" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L23" r:id="rId38" display="App Mech Ground Floor Seminar Hall.jpg"/>
-    <hyperlink ref="Q23" r:id="rId39" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q23" r:id="rId39" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L24" r:id="rId40" display="R22.jpg"/>
-    <hyperlink ref="Q24" r:id="rId41" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q24" r:id="rId41" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L25" r:id="rId42" display="https://drive.google.com/file/d/11r8JUGcdvTO0ylOI_nn1YEYv9b4CKOKq/view?usp=sharing"/>
-    <hyperlink ref="Q25" r:id="rId43" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q25" r:id="rId43" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L26" r:id="rId44" display="https://drive.google.com/file/d/1xfCJ7OavNoyQdfRC-VI19CAZpL4tOAEL/view?usp=sharing"/>
-    <hyperlink ref="Q26" r:id="rId45" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q26" r:id="rId45" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L27" r:id="rId46" display="https://drive.google.com/file/d/1WSBvMorlthEbWyaCh8JdxRMas7G4kjVu/view?usp=sharing"/>
-    <hyperlink ref="Q27" r:id="rId47" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q28" r:id="rId48" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q27" r:id="rId47" display="hod.mech@coeptech.ac.in"/>
+    <hyperlink ref="Q28" r:id="rId48" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L29" r:id="rId49" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
-    <hyperlink ref="Q29" r:id="rId50" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q29" r:id="rId50" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L30" r:id="rId51" display="https://drive.google.com/file/d/1E-q97N6HQpt942F05ddKGT_D6nsHbDe_/view?usp=sharing"/>
-    <hyperlink ref="Q30" r:id="rId52" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q30" r:id="rId52" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L31" r:id="rId53" display="https://drive.google.com/file/d/1orGoTWToL2cNbFSvNjVnGiJBTqj4-x7p/view?usp=sharing"/>
-    <hyperlink ref="Q31" r:id="rId54" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q31" r:id="rId54" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L32" r:id="rId55" display="https://drive.google.com/file/d/1bJecDqhyMaVv0s9jZLgIDUpY1PGb-2qw/view?usp=sharing"/>
-    <hyperlink ref="Q32" r:id="rId56" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q32" r:id="rId56" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L33" r:id="rId57" display="https://drive.google.com/file/d/1zkM7jOLKgqLJAzCTxcQH-GfV_CBt2ZKh/view?usp=sharing"/>
-    <hyperlink ref="Q33" r:id="rId58" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q33" r:id="rId58" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L34" r:id="rId59" display="https://drive.google.com/file/d/1V56Qmp1d-mKg5U3SGllOvQp56yiec8hE/view?usp=sharing"/>
-    <hyperlink ref="Q34" r:id="rId60" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q34" r:id="rId60" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L35" r:id="rId61" display="https://drive.google.com/file/d/1pcndMBRukVQKbKa81_jG_82Q2cZywHFu/view?usp=sharing"/>
-    <hyperlink ref="Q35" r:id="rId62" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q35" r:id="rId62" display="hod.mech@coeptech.ac.in"/>
     <hyperlink ref="L36" r:id="rId63" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="Q36" r:id="rId64" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q36" r:id="rId64" display="hod.elec@coeptech.ac.in"/>
     <hyperlink ref="L37" r:id="rId65" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="Q37" r:id="rId66" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q37" r:id="rId66" display="hod.elec@coeptech.ac.in"/>
     <hyperlink ref="L38" r:id="rId67" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="Q38" r:id="rId68" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q38" r:id="rId68" display="hod.elec@coeptech.ac.in"/>
     <hyperlink ref="L39" r:id="rId69" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="Q39" r:id="rId70" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q39" r:id="rId70" display="hod.elec@coeptech.ac.in"/>
     <hyperlink ref="L40" r:id="rId71" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="Q40" r:id="rId72" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q40" r:id="rId72" display="hod.elec@coeptech.ac.in"/>
     <hyperlink ref="L41" r:id="rId73" display="EED Classrooms_ 24 4 2025"/>
-    <hyperlink ref="Q41" r:id="rId74" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q42" r:id="rId75" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q41" r:id="rId74" display="hod.elec@coeptech.ac.in"/>
+    <hyperlink ref="Q42" r:id="rId75" display="hod.civil@coeptech.ac.in"/>
     <hyperlink ref="L43" r:id="rId76" display="Env Classroom.jpeg"/>
-    <hyperlink ref="Q43" r:id="rId77" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q43" r:id="rId77" display="hod.civil@coeptech.ac.in"/>
     <hyperlink ref="L44" r:id="rId78" display="CM Classroom.jpeg"/>
-    <hyperlink ref="Q44" r:id="rId79" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q45" r:id="rId80" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q44" r:id="rId79" display="hod.civil@coeptech.ac.in"/>
+    <hyperlink ref="Q45" r:id="rId80" display="hod.civil@coeptech.ac.in"/>
     <hyperlink ref="L46" r:id="rId81" display="R8.jpeg"/>
-    <hyperlink ref="Q46" r:id="rId82" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q46" r:id="rId82" display="hod.civil@coeptech.ac.in"/>
     <hyperlink ref="L47" r:id="rId83" display="Geotech Classroom.jpeg"/>
-    <hyperlink ref="Q47" r:id="rId84" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q48" r:id="rId85" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q49" r:id="rId86" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q50" r:id="rId87" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q51" r:id="rId88" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q52" r:id="rId89" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q53" r:id="rId90" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q54" r:id="rId91" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q55" r:id="rId92" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q56" r:id="rId93" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q57" r:id="rId94" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q58" r:id="rId95" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q59" r:id="rId96" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q60" r:id="rId97" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q61" r:id="rId98" display="dean.engineering@coeptech.ac.in"/>
-    <hyperlink ref="Q62" r:id="rId99" display="dean.engineering@coeptech.ac.in"/>
+    <hyperlink ref="Q47" r:id="rId84" display="hod.civil@coeptech.ac.in"/>
+    <hyperlink ref="Q48" r:id="rId85" display="hod.prod@coeptech.ac.in"/>
+    <hyperlink ref="Q49" r:id="rId86" display="hod.prod@coeptech.ac.in"/>
+    <hyperlink ref="Q50" r:id="rId87" display="hod.prod@coeptech.ac.in"/>
+    <hyperlink ref="Q51" r:id="rId88" display="hod.prod@coeptech.ac.in"/>
+    <hyperlink ref="Q52" r:id="rId89" display="hod.prod@coeptech.ac.in"/>
+    <hyperlink ref="Q53" r:id="rId90" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q54" r:id="rId91" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q55" r:id="rId92" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q56" r:id="rId93" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q57" r:id="rId94" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q58" r:id="rId95" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q59" r:id="rId96" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q60" r:id="rId97" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q61" r:id="rId98" display="hod.meta@coeptech.ac.in"/>
+    <hyperlink ref="Q62" r:id="rId99" display="hod.meta@coeptech.ac.in"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>